<commit_message>
pour publication 1.0.1 (#78)
* pour publication 1.0.1

* Update sushi-config.yaml

* Update publication-request.json

* Update publication-request.json

* Update publication-request.json

* Update sushi-config.yaml 8031a1e9ed9bb9603fbd108410b0fc6e016c9a58
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-tddui-bundle.xlsx
+++ b/main/ig/StructureDefinition-tddui-bundle.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.0.1-ballot</t>
+    <t>1.0.1</t>
   </si>
   <si>
     <t>Name</t>
@@ -48,7 +48,7 @@
     <t>Status</t>
   </si>
   <si>
-    <t>draft</t>
+    <t>active</t>
   </si>
   <si>
     <t>Experimental</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-03-29T13:14:00+00:00</t>
+    <t>2024-03-29T13:28:39+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Description fonctionnelle des ressources : Evenement Evaluation (#146)
* Evaluation

* Description des classes tddui

* Update bloc_identification_coordonnees.plantuml

* issue 129

* Issue 129 Statut

* Update donnees_admin.plantuml

* corr sfe issue 129 1ade3700335413ea8410978f6c6a4c11db31e064
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-tddui-bundle.xlsx
+++ b/main/ig/StructureDefinition-tddui-bundle.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-09-06T13:26:49+00:00</t>
+    <t>2024-09-23T13:29:51+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -619,7 +619,7 @@
 * Results from operations might involve resources that are not identified.</t>
   </si>
   <si>
-    <t>fullUrl might not be [unique in the context of a resource](bundle.html#bundle-unique). Note that since [FHIR resources do not need to be served through the FHIR API](http://hl7.org/fhir/R4/references.html), the fullURL might be a URN or an absolute URL that does not end with the logical id of the resource (Resource.id). However, but if the fullUrl does look like a RESTful server URL (e.g. meets the [regex](http://hl7.org/fhir/R4/references.html#regex), then the 'id' portion of the fullUrl SHALL end with the Resource.id.
+    <t>fullUrl might not be [unique in the context of a resource](http://hl7.org/fhir/R4/bundle.html#bundle-unique). Note that since [FHIR resources do not need to be served through the FHIR API](http://hl7.org/fhir/R4/references.html), the fullURL might be a URN or an absolute URL that does not end with the logical id of the resource (Resource.id). However, but if the fullUrl does look like a RESTful server URL (e.g. meets the [regex](http://hl7.org/fhir/R4/references.html#regex), then the 'id' portion of the fullUrl SHALL end with the Resource.id.
 Note that the fullUrl is not the same as the canonical URL - it's an absolute url for an endpoint serving the resource (these will happen to have the same value on the canonical server for the resource with the canonical URL).</t>
   </si>
   <si>

</xml_diff>

<commit_message>
ANS-006-168 - Contact (#424)
* ajout contact

* upate contact

* TDDUIRelatedPerson

* update mapping

* correction

* update VS

* fix

* Ajout JDV-J384

* update contact

* maj VS

* maj instance 20812f7661c4f158d763c7e541d5269ba6838e64
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-tddui-bundle.xlsx
+++ b/main/ig/StructureDefinition-tddui-bundle.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-02-05T13:38:35+00:00</t>
+    <t>2026-02-05T14:50:20+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -3133,34 +3133,34 @@
     <t>Bundle.entry:DUITaskPrestation.response.outcome</t>
   </si>
   <si>
-    <t>Bundle.entry:RelatedPerson</t>
-  </si>
-  <si>
-    <t>RelatedPerson</t>
-  </si>
-  <si>
-    <t>RelatedPerson conforming to the FrCoreRelatedPerson profile, used to convey information about the user's contacts.</t>
-  </si>
-  <si>
-    <t>Bundle.entry:RelatedPerson.id</t>
-  </si>
-  <si>
-    <t>Bundle.entry:RelatedPerson.extension</t>
-  </si>
-  <si>
-    <t>Bundle.entry:RelatedPerson.modifierExtension</t>
-  </si>
-  <si>
-    <t>Bundle.entry:RelatedPerson.link</t>
-  </si>
-  <si>
-    <t>Bundle.entry:RelatedPerson.fullUrl</t>
-  </si>
-  <si>
-    <t>Bundle.entry:RelatedPerson.resource</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RelatedPerson {https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-related-person}
+    <t>Bundle.entry:DUIRelatedPersonContact</t>
+  </si>
+  <si>
+    <t>DUIRelatedPersonContact</t>
+  </si>
+  <si>
+    <t>RelatedPerson conforming to the TDDUIRelatedPersonContact profile, used to convey information about the contact person.</t>
+  </si>
+  <si>
+    <t>Bundle.entry:DUIRelatedPersonContact.id</t>
+  </si>
+  <si>
+    <t>Bundle.entry:DUIRelatedPersonContact.extension</t>
+  </si>
+  <si>
+    <t>Bundle.entry:DUIRelatedPersonContact.modifierExtension</t>
+  </si>
+  <si>
+    <t>Bundle.entry:DUIRelatedPersonContact.link</t>
+  </si>
+  <si>
+    <t>Bundle.entry:DUIRelatedPersonContact.fullUrl</t>
+  </si>
+  <si>
+    <t>Bundle.entry:DUIRelatedPersonContact.resource</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RelatedPerson {https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-related-person-contact}
 </t>
   </si>
   <si>
@@ -3173,79 +3173,79 @@
     <t>role</t>
   </si>
   <si>
-    <t>Bundle.entry:RelatedPerson.search</t>
-  </si>
-  <si>
-    <t>Bundle.entry:RelatedPerson.search.id</t>
-  </si>
-  <si>
-    <t>Bundle.entry:RelatedPerson.search.extension</t>
-  </si>
-  <si>
-    <t>Bundle.entry:RelatedPerson.search.modifierExtension</t>
-  </si>
-  <si>
-    <t>Bundle.entry:RelatedPerson.search.mode</t>
-  </si>
-  <si>
-    <t>Bundle.entry:RelatedPerson.search.score</t>
-  </si>
-  <si>
-    <t>Bundle.entry:RelatedPerson.request</t>
-  </si>
-  <si>
-    <t>Bundle.entry:RelatedPerson.request.id</t>
-  </si>
-  <si>
-    <t>Bundle.entry:RelatedPerson.request.extension</t>
-  </si>
-  <si>
-    <t>Bundle.entry:RelatedPerson.request.modifierExtension</t>
-  </si>
-  <si>
-    <t>Bundle.entry:RelatedPerson.request.method</t>
-  </si>
-  <si>
-    <t>Bundle.entry:RelatedPerson.request.url</t>
-  </si>
-  <si>
-    <t>Bundle.entry:RelatedPerson.request.ifNoneMatch</t>
-  </si>
-  <si>
-    <t>Bundle.entry:RelatedPerson.request.ifModifiedSince</t>
-  </si>
-  <si>
-    <t>Bundle.entry:RelatedPerson.request.ifMatch</t>
-  </si>
-  <si>
-    <t>Bundle.entry:RelatedPerson.request.ifNoneExist</t>
-  </si>
-  <si>
-    <t>Bundle.entry:RelatedPerson.response</t>
-  </si>
-  <si>
-    <t>Bundle.entry:RelatedPerson.response.id</t>
-  </si>
-  <si>
-    <t>Bundle.entry:RelatedPerson.response.extension</t>
-  </si>
-  <si>
-    <t>Bundle.entry:RelatedPerson.response.modifierExtension</t>
-  </si>
-  <si>
-    <t>Bundle.entry:RelatedPerson.response.status</t>
-  </si>
-  <si>
-    <t>Bundle.entry:RelatedPerson.response.location</t>
-  </si>
-  <si>
-    <t>Bundle.entry:RelatedPerson.response.etag</t>
-  </si>
-  <si>
-    <t>Bundle.entry:RelatedPerson.response.lastModified</t>
-  </si>
-  <si>
-    <t>Bundle.entry:RelatedPerson.response.outcome</t>
+    <t>Bundle.entry:DUIRelatedPersonContact.search</t>
+  </si>
+  <si>
+    <t>Bundle.entry:DUIRelatedPersonContact.search.id</t>
+  </si>
+  <si>
+    <t>Bundle.entry:DUIRelatedPersonContact.search.extension</t>
+  </si>
+  <si>
+    <t>Bundle.entry:DUIRelatedPersonContact.search.modifierExtension</t>
+  </si>
+  <si>
+    <t>Bundle.entry:DUIRelatedPersonContact.search.mode</t>
+  </si>
+  <si>
+    <t>Bundle.entry:DUIRelatedPersonContact.search.score</t>
+  </si>
+  <si>
+    <t>Bundle.entry:DUIRelatedPersonContact.request</t>
+  </si>
+  <si>
+    <t>Bundle.entry:DUIRelatedPersonContact.request.id</t>
+  </si>
+  <si>
+    <t>Bundle.entry:DUIRelatedPersonContact.request.extension</t>
+  </si>
+  <si>
+    <t>Bundle.entry:DUIRelatedPersonContact.request.modifierExtension</t>
+  </si>
+  <si>
+    <t>Bundle.entry:DUIRelatedPersonContact.request.method</t>
+  </si>
+  <si>
+    <t>Bundle.entry:DUIRelatedPersonContact.request.url</t>
+  </si>
+  <si>
+    <t>Bundle.entry:DUIRelatedPersonContact.request.ifNoneMatch</t>
+  </si>
+  <si>
+    <t>Bundle.entry:DUIRelatedPersonContact.request.ifModifiedSince</t>
+  </si>
+  <si>
+    <t>Bundle.entry:DUIRelatedPersonContact.request.ifMatch</t>
+  </si>
+  <si>
+    <t>Bundle.entry:DUIRelatedPersonContact.request.ifNoneExist</t>
+  </si>
+  <si>
+    <t>Bundle.entry:DUIRelatedPersonContact.response</t>
+  </si>
+  <si>
+    <t>Bundle.entry:DUIRelatedPersonContact.response.id</t>
+  </si>
+  <si>
+    <t>Bundle.entry:DUIRelatedPersonContact.response.extension</t>
+  </si>
+  <si>
+    <t>Bundle.entry:DUIRelatedPersonContact.response.modifierExtension</t>
+  </si>
+  <si>
+    <t>Bundle.entry:DUIRelatedPersonContact.response.status</t>
+  </si>
+  <si>
+    <t>Bundle.entry:DUIRelatedPersonContact.response.location</t>
+  </si>
+  <si>
+    <t>Bundle.entry:DUIRelatedPersonContact.response.etag</t>
+  </si>
+  <si>
+    <t>Bundle.entry:DUIRelatedPersonContact.response.lastModified</t>
+  </si>
+  <si>
+    <t>Bundle.entry:DUIRelatedPersonContact.response.outcome</t>
   </si>
   <si>
     <t>Bundle.signature</t>

</xml_diff>